<commit_message>
feat: update .gitignore and add AGENTS.md for QA instructions
</commit_message>
<xml_diff>
--- a/Pengujian UNI-NEXUS.xlsx
+++ b/Pengujian UNI-NEXUS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\College\Telkom University\Associate Degree of Information Systems\Projects\UNI-NEXUS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3284A4DC-995E-4C2A-858A-8A59831C9386}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E92382A-4A66-4F4E-A6CC-B69FFE6282D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1567" uniqueCount="1430">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1575" uniqueCount="1434">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -9690,6 +9690,18 @@
 • Global Search tidak pernah menjadi bypass permission/workspace.
 • Debounce+Abort mencegah stale result race dan keyboard interaction dapat digunakan penuh.
 • Dengan kasus ini, seluruh fitur global production yang ditemukan final route audit memiliki coverage eksplisit.</t>
+  </si>
+  <si>
+    <t>[2026-09-14 16:17 WIB] Dry run oleh ACCOUNT #4 (Chief Technology Officer). Currency IDR -&gt; USD: dialog 'Ubah mata uang default?' tampil dengan penjelasan dampak; Batal tidak mengubah nilai setelah reload, konfirmasi menyimpan USD, lalu nilai berhasil dipulihkan ke IDR. Timezone Asia/Jakarta -&gt; UTC: dialog 'Ubah zona waktu organisasi?' tampil dengan penjelasan bahwa timestamp historis tidak ditulis ulang; setelah 'Simpan Zona Waktu', alert 'Data pengaturan tidak valid.' tampil, nilai UTC tidak persisten, dan browser mencatat respons HTTP 400 pada /api/v1/settings/organization. Langkah lanjutan timezone dan uji gabungan tidak dilanjutkan karena kegagalan ini. Nilai asli Currency IDR dan Timezone Asia/Jakarta dipulihkan serta diverifikasi setelah reload. Tidak ada transaksi/dokumen historis tersedia di UI untuk verifikasi konversi/timestamp. Bukti: test-evidence/dry-run-1/UNX-S03-003/timezone-save-failure.png.</t>
+  </si>
+  <si>
+    <t>Dry Run 2 2026-09-14: Diuji via frontend. CTO melihat 7 dataset dan kontrol kelola; Insinyur 3D melihat 6 dataset sesuai scope tanpa Tambah Data/Kelola. Blocked pada langkah Penggunaan karena semua dataset berisi 0 record sehingga aksi Penggunaan pada record tidak tersedia. Status dibiarkan kosong karena dropdown hanya Pass/Bug/Failed. Bukti: test-evidence/dry-run-2/UNX-S03-008/01-cto-initial-state.png dan 02-engineer-read-only.png.</t>
+  </si>
+  <si>
+    <t>Dry Run 2 2026-09-14: Diuji via frontend. Navigasi 7 dataset, pencarian, filter, refresh, dan viewport mobile tanpa overflow terverifikasi. Blocked untuk filter yang menghasilkan data, pagination &gt;25, dan ekspor CSV/XLSX nonkosong karena seluruh dataset berisi 0 record. Status dibiarkan kosong karena dropdown hanya Pass/Bug/Failed. Bukti: test-evidence/dry-run-2/UNX-S03-009/01-initial-overview.png dan 03-mobile-empty-state.png.</t>
+  </si>
+  <si>
+    <t>Dry Run 2 2026-09-14: Pass. QA_U_163552 dibuat aktif dan diedit menjadi Satuan QA Edit 163552 (qe, weight, 3 desimal). Validasi input, uppercase, duplicate, code lock, penggunaan 0, batal nonaktif, nonaktif/aktif kembali terverifikasi. Satuan QA dibiarkan aktif untuk prasyarat test lanjutan. Bukti: test-evidence/dry-run-2/UNX-S03-010/01-validation-error.png dan 02-final-active-unit.png.</t>
   </si>
 </sst>
 </file>
@@ -11210,9 +11222,13 @@
       <c r="E34" s="4" t="s">
         <v>188</v>
       </c>
-      <c r="F34" s="5"/>
+      <c r="F34" s="5" t="s">
+        <v>58</v>
+      </c>
       <c r="G34" s="4"/>
-      <c r="H34" s="4"/>
+      <c r="H34" s="4" t="s">
+        <v>1430</v>
+      </c>
       <c r="I34" s="4"/>
       <c r="O34" s="10"/>
     </row>
@@ -11328,9 +11344,13 @@
       <c r="E39" s="4" t="s">
         <v>210</v>
       </c>
-      <c r="F39" s="5"/>
+      <c r="F39" s="5" t="s">
+        <v>58</v>
+      </c>
       <c r="G39" s="4"/>
-      <c r="H39" s="4"/>
+      <c r="H39" s="4" t="s">
+        <v>1431</v>
+      </c>
       <c r="I39" s="4"/>
       <c r="O39" s="10"/>
     </row>
@@ -11350,9 +11370,13 @@
       <c r="E40" s="4" t="s">
         <v>215</v>
       </c>
-      <c r="F40" s="5"/>
+      <c r="F40" s="5" t="s">
+        <v>58</v>
+      </c>
       <c r="G40" s="4"/>
-      <c r="H40" s="4"/>
+      <c r="H40" s="4" t="s">
+        <v>1432</v>
+      </c>
       <c r="I40" s="4"/>
       <c r="O40" s="10"/>
     </row>
@@ -11372,9 +11396,13 @@
       <c r="E41" s="4" t="s">
         <v>220</v>
       </c>
-      <c r="F41" s="5"/>
+      <c r="F41" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="G41" s="4"/>
-      <c r="H41" s="4"/>
+      <c r="H41" s="4" t="s">
+        <v>1433</v>
+      </c>
       <c r="I41" s="4"/>
       <c r="O41" s="10"/>
     </row>

</xml_diff>